<commit_message>
Añadí lo del trafico, puse max heap para prioridades de atención
</commit_message>
<xml_diff>
--- a/datos/capacidades.xlsx
+++ b/datos/capacidades.xlsx
@@ -472,10 +472,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -495,10 +495,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -518,10 +518,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
         <v>10</v>
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
         <v>4</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -610,10 +610,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -633,10 +633,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -656,10 +656,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -725,10 +725,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -748,10 +748,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -771,10 +771,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -794,10 +794,10 @@
         </is>
       </c>
       <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
         <v>7</v>
-      </c>
-      <c r="E16" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -817,10 +817,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -840,10 +840,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
@@ -863,10 +863,10 @@
         </is>
       </c>
       <c r="D19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" t="n">
         <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -886,10 +886,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -909,10 +909,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -978,10 +978,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1004,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1024,10 +1024,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -1047,10 +1047,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
@@ -1116,10 +1116,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -1135,10 +1135,10 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
@@ -1154,10 +1154,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
@@ -1173,10 +1173,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -1192,10 +1192,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -1218,7 +1218,7 @@
         <v>6</v>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1238,10 +1238,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
@@ -1284,10 +1284,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1330,10 +1330,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E40" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -1353,10 +1353,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -1376,10 +1376,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E42" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -1445,10 +1445,10 @@
         </is>
       </c>
       <c r="D45" t="n">
+        <v>15</v>
+      </c>
+      <c r="E45" t="n">
         <v>5</v>
-      </c>
-      <c r="E45" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="46">
@@ -1468,10 +1468,10 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1487,10 +1487,10 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -1509,7 +1509,7 @@
         <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1525,10 +1525,10 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1567,10 +1567,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E52" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -1613,10 +1613,10 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">
@@ -1636,10 +1636,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55">
@@ -1659,10 +1659,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56">
@@ -1682,10 +1682,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -1705,10 +1705,10 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
@@ -1728,10 +1728,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambios para la visualización en mapa
</commit_message>
<xml_diff>
--- a/datos/capacidades.xlsx
+++ b/datos/capacidades.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,27 +417,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id_hospital</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>especialidad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>camas_totales</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>camas_ocupadas</t>
         </is>
@@ -472,10 +460,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -498,7 +486,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -518,10 +506,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -541,10 +529,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -564,10 +552,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -587,10 +575,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -610,10 +598,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -633,10 +621,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -659,7 +647,7 @@
         <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -682,7 +670,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -702,10 +690,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -725,10 +713,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -748,10 +736,10 @@
         </is>
       </c>
       <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
         <v>8</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -771,10 +759,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -794,7 +782,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E16" t="n">
         <v>7</v>
@@ -817,10 +805,10 @@
         </is>
       </c>
       <c r="D17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" t="n">
         <v>6</v>
-      </c>
-      <c r="E17" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -840,10 +828,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -863,10 +851,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -886,10 +874,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -909,10 +897,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -935,7 +923,7 @@
         <v>13</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -955,10 +943,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -978,7 +966,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -1001,10 +989,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -1024,7 +1012,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>7</v>
@@ -1047,10 +1035,10 @@
         </is>
       </c>
       <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
         <v>4</v>
-      </c>
-      <c r="E27" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -1070,10 +1058,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1093,10 +1081,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
@@ -1116,10 +1104,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -1135,10 +1123,10 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1154,10 +1142,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1173,10 +1161,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -1192,10 +1180,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E34" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -1215,10 +1203,10 @@
         </is>
       </c>
       <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="n">
         <v>6</v>
-      </c>
-      <c r="E35" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1238,10 +1226,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
@@ -1261,10 +1249,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -1284,10 +1272,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E38" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -1307,10 +1295,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -1330,10 +1318,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
@@ -1353,10 +1341,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -1376,10 +1364,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -1399,10 +1387,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44">
@@ -1422,10 +1410,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -1445,10 +1433,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -1468,10 +1456,10 @@
         </is>
       </c>
       <c r="D46" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" t="n">
         <v>6</v>
-      </c>
-      <c r="E46" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1487,10 +1475,10 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
@@ -1506,10 +1494,10 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49">
@@ -1525,10 +1513,10 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -1544,10 +1532,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -1567,10 +1555,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -1590,10 +1578,10 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -1613,10 +1601,10 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -1636,10 +1624,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E54" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1659,10 +1647,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56">
@@ -1682,10 +1670,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57">
@@ -1705,10 +1693,10 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58">
@@ -1728,10 +1716,10 @@
         </is>
       </c>
       <c r="D58" t="n">
+        <v>6</v>
+      </c>
+      <c r="E58" t="n">
         <v>7</v>
-      </c>
-      <c r="E58" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>